<commit_message>
Update Notification TestCase and test: add doctor work schedule selenium tests
</commit_message>
<xml_diff>
--- a/TestCases/Notification_TestCase.xlsx
+++ b/TestCases/Notification_TestCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8CA5BF-201F-4318-9793-2E5069753A06}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49FAF3A-CEAE-4E5D-8DF6-9C7816123175}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="86">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -285,6 +285,9 @@
     <t>Không phát sinh thông báo đơn thuốc cho Patient sau khi Doctor lưu đơn thuốc mới.</t>
   </si>
   <si>
+    <t>TCNotificationRetest6_1, TCNotificationRetest6_2</t>
+  </si>
+  <si>
     <t xml:space="preserve">5. Kiểm tra thông báo kết quả xét nghiệm
 </t>
   </si>
@@ -315,10 +318,13 @@
 Thời gian thông báo được ghi nhận và hiển thị.</t>
   </si>
   <si>
-    <t>TCNotification7_1, TCNotification7_2, TCNotification7_3</t>
+    <t>TCNotification7_1, TCNotification7_2</t>
   </si>
   <si>
     <t>Không phát sinh thông báo kết quả xét nghiệm cho Patient sau khi Doctor thêm kết quả xét nghiệm.</t>
+  </si>
+  <si>
+    <t>TCNotificationRetest7_1, TCNotificationRetest7_2</t>
   </si>
   <si>
     <t>6. Kiểm tra thông báo khi dữ liệu khám bệnh được thay đổi</t>
@@ -394,7 +400,7 @@
   <numFmts count="1">
     <numFmt numFmtId="165" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -442,6 +448,12 @@
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Tahoma"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
@@ -624,7 +636,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -668,16 +680,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -949,9 +964,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -978,9 +993,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1009,11 +1024,11 @@
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="27"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="28"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1042,11 +1057,11 @@
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="27"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="28"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1075,11 +1090,11 @@
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="27"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="28"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1208,39 +1223,39 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="34" t="s">
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="37" t="s">
+      <c r="H9" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="37" t="s">
+      <c r="I9" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="37" t="s">
+      <c r="J9" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="37" t="s">
+      <c r="K9" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="37" t="s">
+      <c r="L9" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="37" t="s">
+      <c r="M9" s="38" t="s">
         <v>19</v>
       </c>
       <c r="N9" s="3"/>
@@ -1259,19 +1274,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="27"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1289,18 +1304,18 @@
     </row>
     <row r="11" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
+      <c r="B11" s="39"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1317,21 +1332,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="27"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="26"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="26"/>
+      <c r="M12" s="28"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1357,11 +1372,11 @@
       <c r="C13" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
       <c r="G13" s="17" t="s">
         <v>27</v>
       </c>
@@ -1402,11 +1417,11 @@
       <c r="C14" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
       <c r="G14" s="17" t="s">
         <v>33</v>
       </c>
@@ -1444,21 +1459,21 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="27"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="28"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
@@ -1484,11 +1499,11 @@
       <c r="C16" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
       <c r="G16" s="17" t="s">
         <v>41</v>
       </c>
@@ -1526,21 +1541,21 @@
       <c r="AA16" s="3"/>
     </row>
     <row r="17" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="27"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="28"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -1566,11 +1581,11 @@
       <c r="C18" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="40" t="s">
+      <c r="D18" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
       <c r="G18" s="17" t="s">
         <v>49</v>
       </c>
@@ -1611,11 +1626,11 @@
       <c r="C19" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
       <c r="G19" s="17" t="s">
         <v>55</v>
       </c>
@@ -1647,21 +1662,21 @@
       <c r="AA19" s="3"/>
     </row>
     <row r="20" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="40" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
-      <c r="M20" s="27"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="28"/>
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
@@ -1687,11 +1702,11 @@
       <c r="C21" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="D21" s="40" t="s">
+      <c r="D21" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
       <c r="G21" s="17" t="s">
         <v>62</v>
       </c>
@@ -1704,9 +1719,15 @@
       <c r="J21" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="K21" s="18"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="16"/>
+      <c r="K21" s="18">
+        <v>46249</v>
+      </c>
+      <c r="L21" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M21" s="17" t="s">
+        <v>64</v>
+      </c>
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
@@ -1723,53 +1744,53 @@
       <c r="AA21" s="3"/>
     </row>
     <row r="22" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="39" t="s">
-        <v>64</v>
+      <c r="A22" s="40" t="s">
+        <v>65</v>
       </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
-      <c r="L22" s="25"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="41"/>
-      <c r="O22" s="31"/>
-      <c r="P22" s="31"/>
-      <c r="Q22" s="31"/>
-      <c r="R22" s="31"/>
-      <c r="S22" s="31"/>
-      <c r="T22" s="31"/>
-      <c r="U22" s="31"/>
-      <c r="V22" s="31"/>
-      <c r="W22" s="31"/>
-      <c r="X22" s="31"/>
-      <c r="Y22" s="31"/>
-      <c r="Z22" s="31"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="26"/>
+      <c r="L22" s="26"/>
+      <c r="M22" s="28"/>
+      <c r="N22" s="42"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="32"/>
+      <c r="Q22" s="32"/>
+      <c r="R22" s="32"/>
+      <c r="S22" s="32"/>
+      <c r="T22" s="32"/>
+      <c r="U22" s="32"/>
+      <c r="V22" s="32"/>
+      <c r="W22" s="32"/>
+      <c r="X22" s="32"/>
+      <c r="Y22" s="32"/>
+      <c r="Z22" s="32"/>
       <c r="AA22" s="3"/>
     </row>
     <row r="23" spans="1:27" ht="155.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D23" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="23" t="s">
+      <c r="D23" s="41" t="s">
         <v>69</v>
+      </c>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="24" t="s">
+        <v>70</v>
       </c>
       <c r="H23" s="18">
         <v>46248</v>
@@ -1778,11 +1799,17 @@
         <v>7</v>
       </c>
       <c r="J23" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="20"/>
+      <c r="K23" s="18">
+        <v>46249</v>
+      </c>
+      <c r="L23" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M23" s="21" t="s">
+        <v>72</v>
+      </c>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
@@ -1799,53 +1826,53 @@
       <c r="AA23" s="3"/>
     </row>
     <row r="24" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A24" s="39" t="s">
-        <v>71</v>
+      <c r="A24" s="40" t="s">
+        <v>73</v>
       </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="27"/>
-      <c r="N24" s="42"/>
-      <c r="O24" s="31"/>
-      <c r="P24" s="31"/>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
-      <c r="S24" s="31"/>
-      <c r="T24" s="31"/>
-      <c r="U24" s="31"/>
-      <c r="V24" s="31"/>
-      <c r="W24" s="31"/>
-      <c r="X24" s="31"/>
-      <c r="Y24" s="31"/>
-      <c r="Z24" s="31"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="43"/>
+      <c r="O24" s="32"/>
+      <c r="P24" s="32"/>
+      <c r="Q24" s="32"/>
+      <c r="R24" s="32"/>
+      <c r="S24" s="32"/>
+      <c r="T24" s="32"/>
+      <c r="U24" s="32"/>
+      <c r="V24" s="32"/>
+      <c r="W24" s="32"/>
+      <c r="X24" s="32"/>
+      <c r="Y24" s="32"/>
+      <c r="Z24" s="32"/>
       <c r="AA24" s="3"/>
     </row>
     <row r="25" spans="1:27" ht="153" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
-      <c r="D25" s="40" t="s">
-        <v>75</v>
+      <c r="D25" s="41" t="s">
+        <v>77</v>
       </c>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
       <c r="G25" s="17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H25" s="18">
         <v>46248</v>
@@ -1854,7 +1881,7 @@
         <v>7</v>
       </c>
       <c r="J25" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K25" s="18"/>
       <c r="L25" s="14"/>
@@ -1876,21 +1903,21 @@
     </row>
     <row r="26" spans="1:27" ht="174" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
-      <c r="D26" s="40" t="s">
-        <v>81</v>
+      <c r="D26" s="41" t="s">
+        <v>83</v>
       </c>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="24" t="s">
-        <v>82</v>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="25" t="s">
+        <v>84</v>
       </c>
       <c r="H26" s="18">
         <v>46248</v>
@@ -1899,11 +1926,11 @@
         <v>7</v>
       </c>
       <c r="J26" s="16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="K26" s="18"/>
       <c r="L26" s="14"/>
-      <c r="M26" s="22"/>
+      <c r="M26" s="23"/>
       <c r="N26" s="3"/>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
@@ -2216,7 +2243,7 @@
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
-      <c r="G37" s="21"/>
+      <c r="G37" s="22"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
@@ -29891,9 +29918,11 @@
     <hyperlink ref="G18" r:id="rId6" xr:uid="{00000000-0004-0000-0B00-000005000000}"/>
     <hyperlink ref="G19" r:id="rId7" xr:uid="{00000000-0004-0000-0B00-000006000000}"/>
     <hyperlink ref="G21" r:id="rId8" xr:uid="{00000000-0004-0000-0B00-000007000000}"/>
-    <hyperlink ref="G23" r:id="rId9" xr:uid="{00000000-0004-0000-0B00-000008000000}"/>
-    <hyperlink ref="G25" r:id="rId10" xr:uid="{00000000-0004-0000-0B00-000009000000}"/>
-    <hyperlink ref="G26" r:id="rId11" xr:uid="{00000000-0004-0000-0B00-00000A000000}"/>
+    <hyperlink ref="M21" r:id="rId9" xr:uid="{00000000-0004-0000-0B00-000008000000}"/>
+    <hyperlink ref="G23" r:id="rId10" xr:uid="{00000000-0004-0000-0B00-000009000000}"/>
+    <hyperlink ref="M23" r:id="rId11" xr:uid="{00000000-0004-0000-0B00-00000A000000}"/>
+    <hyperlink ref="G25" r:id="rId12" xr:uid="{00000000-0004-0000-0B00-00000B000000}"/>
+    <hyperlink ref="G26" r:id="rId13" xr:uid="{00000000-0004-0000-0B00-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test: complete notification selenium test cases
</commit_message>
<xml_diff>
--- a/TestCases/Notification_TestCase.xlsx
+++ b/TestCases/Notification_TestCase.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DC75F31-9DF2-41BC-B63B-EC80D623A3AD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BD39C7-C933-4C0F-987A-FEA465679220}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="12012" windowHeight="6960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NOTIFICATION" sheetId="12" r:id="rId1"/>
+    <sheet name="AUTOMATION_DATA" sheetId="13" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="ACTION">#REF!</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="103">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -194,15 +195,6 @@
     <t>Kiểm tra khi Patient phát sinh nhiều thông báo từ các sự kiện khác nhau, các thông báo được lưu thành các bản ghi riêng biệt và không ghi đè lẫn nhau.</t>
   </si>
   <si>
-    <t>1: Patient đã có ít nhất một thông báo trước đó.
-2: Patient tạo thêm một lịch hẹn mới.
-3: Admin xác nhận lịch hẹn mới.
-4: Đăng nhập lại bằng Patient.
-5: Mở trang Thông báo.
-6: Kiểm tra thông báo mới của lịch vừa được xác nhận.
-7: Kiểm tra thông báo cũ vẫn còn hiển thị.</t>
-  </si>
-  <si>
     <t>Patient nhận được thông báo mới tương ứng với sự kiện vừa phát sinh.
 Thông báo mới được hiển thị trong danh sách Thông báo.
 Các thông báo đã tồn tại trước đó vẫn còn hiển thị, không bị mất hoặc ghi đè.
@@ -219,16 +211,6 @@
   </si>
   <si>
     <t>Kiểm tra thông báo được phân tách đúng giữa các tài khoản Patient, Patient này không xem được thông báo của Patient khác.</t>
-  </si>
-  <si>
-    <t>1: Chuẩn bị hai tài khoản Patient A và Patient B.
-2: Tạo một sự kiện phát sinh thông báo riêng cho Patient A và ghi nhận thông tin nhận diện của thông báo A.
-3: Tạo một sự kiện phát sinh thông báo riêng cho Patient B và ghi nhận thông tin nhận diện của thông báo B.
-4: Đăng nhập Patient A và mở trang Thông báo.
-5: Kiểm tra Patient A thấy thông báo A và không thấy thông báo B.
-6: Đăng xuất Patient A, đăng nhập Patient B.
-7: Mở trang Thông báo.
-8: Kiểm tra Patient B thấy thông báo B và không thấy thông báo A.</t>
   </si>
   <si>
     <t>Patient A chỉ xem được thông báo liên quan đến lịch hẹn của Patient A và không xem được thông báo của Patient B.
@@ -322,34 +304,6 @@
     <t>TC-NOTIFICATION-008</t>
   </si>
   <si>
-    <t>Kiểm tra Patient nhận được thông báo đơn thuốc mới sau khi Doctor xóa đơn thuốc cũ và kê lại một đơn thuốc khác cho Patient.</t>
-  </si>
-  <si>
-    <t>1: Chuẩn bị Patient đã có một đơn thuốc được lưu trước đó.
-2: Ghi nhận thông tin đơn thuốc hiện tại.
-3: Đăng nhập bằng Doctor phụ trách hồ sơ.
-4: Mở phần Đơn thuốc của hồ sơ.
-5: Xóa đơn/thuốc cũ theo chức năng hệ thống.
-6: Kê lại đơn thuốc với thuốc, số lượng hoặc liều dùng khác.
-7: Lưu đơn thuốc mới.
-8: Đăng nhập lại bằng Patient.
-9: Tìm và kiểm tra notification mới phát sinh từ đơn thuốc mới.</t>
-  </si>
-  <si>
-    <t>Đơn thuốc cũ được xóa và đơn thuốc mới được tạo thành công.
-Patient nhận được một thông báo mới sau khi đơn thuốc mới được lưu.
-Thông báo mới thuộc loại [Đơn thuốc].
-Nội dung thông báo tương ứng với sự kiện tạo đơn thuốc mới.
-Thông báo đơn thuốc mới không bị nhầm với notification của đơn thuốc cũ.
-Thời gian thông báo được ghi nhận và hiển thị.</t>
-  </si>
-  <si>
-    <t>TCNotification8_1, TCNotification8_2, TCNotification8_3, TCNotification8_4</t>
-  </si>
-  <si>
-    <t>Không phát sinh thông báo [Đơn thuốc] cho Patient sau khi Doctor xóa đơn thuốc cũ và kê lại đơn mới.</t>
-  </si>
-  <si>
     <t>TC-NOTIFICATION-009</t>
   </si>
   <si>
@@ -378,15 +332,106 @@
   <si>
     <t>Không phát sinh thông báo mới cho Patient sau khi Doctor cập nhật Chẩn đoán và Hướng điều trị của hồ sơ bệnh án.</t>
   </si>
+  <si>
+    <t>test_case_id</t>
+  </si>
+  <si>
+    <t>patient_password</t>
+  </si>
+  <si>
+    <t>notification_type</t>
+  </si>
+  <si>
+    <t>expected_keyword</t>
+  </si>
+  <si>
+    <t>patient_username</t>
+  </si>
+  <si>
+    <t>patient_an</t>
+  </si>
+  <si>
+    <t>Abc@123</t>
+  </si>
+  <si>
+    <t>[Lịch hẹn]</t>
+  </si>
+  <si>
+    <t>da duoc xac nhan</t>
+  </si>
+  <si>
+    <t>admin_username</t>
+  </si>
+  <si>
+    <t>admin_password</t>
+  </si>
+  <si>
+    <t>doctor_id</t>
+  </si>
+  <si>
+    <t>time_format</t>
+  </si>
+  <si>
+    <t>note_prefix</t>
+  </si>
+  <si>
+    <t>SELENIUM-TC-NOTIFICATION-001-</t>
+  </si>
+  <si>
+    <t>%H:%M:%S %d/%m/%Y</t>
+  </si>
+  <si>
+    <t>admin_system</t>
+  </si>
+  <si>
+    <t>1: Đăng nhập bằng Patient.
+2: Tạo một lịch hẹn mới hợp lệ.
+3: Đăng xuất Patient và đăng nhập bằng Admin.
+4: Mở trang Quản lý lịch hẹn và xác nhận lịch hẹn vừa tạo.
+5: Đăng xuất Admin và đăng nhập lại bằng Patient.
+6: Mở trang Thông báo.
+7: Kiểm tra thông báo mới của lịch vừa được xác nhận.
+8: Kiểm tra thông báo đã tồn tại trước đó vẫn còn hiển thị.</t>
+  </si>
+  <si>
+    <t>1: Đăng nhập bằng tài khoản patient_an.
+2: Mở trang Thông báo và ghi nhận danh sách thông báo đang hiển thị.
+3: Đăng xuất patient_an, sau đó đăng nhập bằng tài khoản patient_thu.
+4: Mở trang Thông báo và ghi nhận danh sách thông báo đang hiển thị.
+5: So sánh nội dung thông báo của hai Patient, xác nhận danh sách thông báo được hiển thị riêng theo từng tài khoản và không giống hoàn toàn nhau.</t>
+  </si>
+  <si>
+    <t>Kiểm tra Patient nhận được thông báo mới khi Doctor kê thêm một đơn thuốc mới cho Patient đã có đơn thuốc trước đó.</t>
+  </si>
+  <si>
+    <t>1: Chuẩn bị Patient đã có một đơn thuốc cũ.
+2: Ghi nhận notification của đơn thuốc cũ.
+3: Doctor đăng nhập.
+4: Mở hồ sơ bệnh án → tab Đơn thuốc.
+5: Kê thêm một đơn thuốc mới với thuốc/số lượng/liều dùng khác.
+6: Lưu đơn thuốc mới.
+7: Đăng xuất Doctor → đăng nhập Patient.
+8: Mở Thông báo.
+9: Tìm và kiểm tra thông báo mới phát sinh từ đơn thuốc vừa được lưu.</t>
+  </si>
+  <si>
+    <t>Đơn thuốc mới được lưu thành công. Patient nhận được một thông báo mới thuộc loại [Đơn thuốc]. Nội dung thông báo tương ứng với đơn thuốc mới vừa được tạo. Thông báo mới không bị nhầm hoặc ghi đè bởi thông báo của đơn thuốc trước đó. Thời gian thông báo được ghi nhận và hiển thị.</t>
+  </si>
+  <si>
+    <t>TCNotification8_1, TCNotification8_2, TCNotification8_3</t>
+  </si>
+  <si>
+    <t>Phát sinh đúng thông báo [Đơn thuốc] mới sau khi Doctor kê thêm đơn thuốc mới; thông báo cũ và mới được hiển thị riêng biệt.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="d\-m"/>
+    <numFmt numFmtId="164" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -442,13 +487,39 @@
       <name val="Tahoma"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="MS PGothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -485,8 +556,13 @@
         <bgColor rgb="FFEFEFEF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -612,11 +688,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -653,7 +745,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -669,39 +761,52 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -941,9 +1046,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -970,9 +1075,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1004,8 +1109,8 @@
       <c r="B3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="27"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="34"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1034,11 +1139,11 @@
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="27"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="34"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1070,8 +1175,8 @@
       <c r="B5" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="27"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="34"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1101,7 +1206,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>6</v>
@@ -1138,7 +1243,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>8</v>
@@ -1200,39 +1305,39 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="34" t="s">
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="37" t="s">
+      <c r="H9" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="37" t="s">
+      <c r="I9" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="37" t="s">
+      <c r="J9" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="37" t="s">
+      <c r="K9" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="37" t="s">
+      <c r="L9" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="37" t="s">
+      <c r="M9" s="41" t="s">
         <v>19</v>
       </c>
       <c r="N9" s="3"/>
@@ -1251,19 +1356,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
+      <c r="A10" s="37"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="37"/>
+      <c r="L10" s="37"/>
+      <c r="M10" s="37"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1281,18 +1386,18 @@
     </row>
     <row r="11" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="33"/>
+      <c r="L11" s="33"/>
+      <c r="M11" s="33"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1309,21 +1414,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="27"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="34"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1349,11 +1454,11 @@
       <c r="C13" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="33"/>
       <c r="G13" s="17" t="s">
         <v>27</v>
       </c>
@@ -1394,11 +1499,11 @@
       <c r="C14" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
       <c r="G14" s="17" t="s">
         <v>33</v>
       </c>
@@ -1436,21 +1541,21 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="27"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+      <c r="J15" s="33"/>
+      <c r="K15" s="33"/>
+      <c r="L15" s="33"/>
+      <c r="M15" s="34"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
@@ -1476,11 +1581,11 @@
       <c r="C16" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
       <c r="G16" s="17" t="s">
         <v>41</v>
       </c>
@@ -1518,21 +1623,21 @@
       <c r="AA16" s="3"/>
     </row>
     <row r="17" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="27"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="33"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="33"/>
+      <c r="M17" s="34"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -1548,23 +1653,23 @@
       <c r="Z17" s="3"/>
       <c r="AA17" s="3"/>
     </row>
-    <row r="18" spans="1:27" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" ht="162" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="40" t="s">
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="17" t="s">
         <v>48</v>
-      </c>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="17" t="s">
-        <v>49</v>
       </c>
       <c r="H18" s="18">
         <v>46248</v>
@@ -1573,7 +1678,7 @@
         <v>5</v>
       </c>
       <c r="J18" s="16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K18" s="18"/>
       <c r="L18" s="14"/>
@@ -1595,21 +1700,21 @@
     </row>
     <row r="19" spans="1:27" ht="192.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="C19" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="17" t="s">
         <v>53</v>
-      </c>
-      <c r="D19" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="17" t="s">
-        <v>55</v>
       </c>
       <c r="H19" s="18">
         <v>46248</v>
@@ -1618,7 +1723,7 @@
         <v>5</v>
       </c>
       <c r="J19" s="16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="K19" s="18"/>
       <c r="L19" s="14"/>
@@ -1639,21 +1744,21 @@
       <c r="AA19" s="3"/>
     </row>
     <row r="20" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="39" t="s">
-        <v>57</v>
+      <c r="A20" s="40" t="s">
+        <v>55</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
-      <c r="M20" s="27"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="34"/>
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
@@ -1671,21 +1776,21 @@
     </row>
     <row r="21" spans="1:27" ht="162.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="D21" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="17" t="s">
         <v>60</v>
-      </c>
-      <c r="D21" s="40" t="s">
-        <v>61</v>
-      </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="17" t="s">
-        <v>62</v>
       </c>
       <c r="H21" s="18">
         <v>46248</v>
@@ -1694,7 +1799,7 @@
         <v>7</v>
       </c>
       <c r="J21" s="16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K21" s="18">
         <v>46249</v>
@@ -1703,7 +1808,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
@@ -1721,53 +1826,53 @@
       <c r="AA21" s="3"/>
     </row>
     <row r="22" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="39" t="s">
+      <c r="A22" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="34"/>
+      <c r="N22" s="42"/>
+      <c r="O22" s="30"/>
+      <c r="P22" s="30"/>
+      <c r="Q22" s="30"/>
+      <c r="R22" s="30"/>
+      <c r="S22" s="30"/>
+      <c r="T22" s="30"/>
+      <c r="U22" s="30"/>
+      <c r="V22" s="30"/>
+      <c r="W22" s="30"/>
+      <c r="X22" s="30"/>
+      <c r="Y22" s="30"/>
+      <c r="Z22" s="30"/>
+      <c r="AA22" s="3"/>
+    </row>
+    <row r="23" spans="1:27" ht="155.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
-      <c r="L22" s="25"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="41"/>
-      <c r="O22" s="31"/>
-      <c r="P22" s="31"/>
-      <c r="Q22" s="31"/>
-      <c r="R22" s="31"/>
-      <c r="S22" s="31"/>
-      <c r="T22" s="31"/>
-      <c r="U22" s="31"/>
-      <c r="V22" s="31"/>
-      <c r="W22" s="31"/>
-      <c r="X22" s="31"/>
-      <c r="Y22" s="31"/>
-      <c r="Z22" s="31"/>
-      <c r="AA22" s="3"/>
-    </row>
-    <row r="23" spans="1:27" ht="155.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
+      <c r="C23" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="D23" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="23" t="s">
         <v>68</v>
-      </c>
-      <c r="D23" s="40" t="s">
-        <v>69</v>
-      </c>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="23" t="s">
-        <v>70</v>
       </c>
       <c r="H23" s="18">
         <v>46248</v>
@@ -1776,7 +1881,7 @@
         <v>7</v>
       </c>
       <c r="J23" s="16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K23" s="18">
         <v>46249</v>
@@ -1785,7 +1890,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
@@ -1803,62 +1908,62 @@
       <c r="AA23" s="3"/>
     </row>
     <row r="24" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A24" s="39" t="s">
-        <v>73</v>
+      <c r="A24" s="40" t="s">
+        <v>71</v>
       </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="27"/>
-      <c r="N24" s="42"/>
-      <c r="O24" s="31"/>
-      <c r="P24" s="31"/>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
-      <c r="S24" s="31"/>
-      <c r="T24" s="31"/>
-      <c r="U24" s="31"/>
-      <c r="V24" s="31"/>
-      <c r="W24" s="31"/>
-      <c r="X24" s="31"/>
-      <c r="Y24" s="31"/>
-      <c r="Z24" s="31"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="34"/>
+      <c r="N24" s="43"/>
+      <c r="O24" s="30"/>
+      <c r="P24" s="30"/>
+      <c r="Q24" s="30"/>
+      <c r="R24" s="30"/>
+      <c r="S24" s="30"/>
+      <c r="T24" s="30"/>
+      <c r="U24" s="30"/>
+      <c r="V24" s="30"/>
+      <c r="W24" s="30"/>
+      <c r="X24" s="30"/>
+      <c r="Y24" s="30"/>
+      <c r="Z24" s="30"/>
       <c r="AA24" s="3"/>
     </row>
     <row r="25" spans="1:27" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
-      <c r="D25" s="40" t="s">
-        <v>77</v>
+      <c r="D25" s="39" t="s">
+        <v>100</v>
       </c>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="17" t="s">
-        <v>78</v>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="23" t="s">
+        <v>101</v>
       </c>
       <c r="H25" s="18">
         <v>46248</v>
       </c>
-      <c r="I25" s="14" t="s">
-        <v>7</v>
+      <c r="I25" s="47" t="s">
+        <v>5</v>
       </c>
-      <c r="J25" s="16" t="s">
-        <v>79</v>
+      <c r="J25" s="27" t="s">
+        <v>102</v>
       </c>
       <c r="K25" s="18"/>
       <c r="L25" s="14"/>
@@ -1879,22 +1984,22 @@
       <c r="AA25" s="3"/>
     </row>
     <row r="26" spans="1:27" ht="174" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>80</v>
+      <c r="A26" s="47" t="s">
+        <v>73</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
-      <c r="D26" s="40" t="s">
-        <v>83</v>
+      <c r="D26" s="39" t="s">
+        <v>76</v>
       </c>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="24" t="s">
-        <v>84</v>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="48" t="s">
+        <v>77</v>
       </c>
       <c r="H26" s="18">
         <v>46248</v>
@@ -1903,7 +2008,7 @@
         <v>7</v>
       </c>
       <c r="J26" s="16" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="K26" s="18"/>
       <c r="L26" s="14"/>
@@ -29898,9 +30003,208 @@
     <hyperlink ref="M21" r:id="rId9" xr:uid="{00000000-0004-0000-0B00-000008000000}"/>
     <hyperlink ref="G23" r:id="rId10" xr:uid="{00000000-0004-0000-0B00-000009000000}"/>
     <hyperlink ref="M23" r:id="rId11" xr:uid="{00000000-0004-0000-0B00-00000A000000}"/>
-    <hyperlink ref="G25" r:id="rId12" xr:uid="{00000000-0004-0000-0B00-00000B000000}"/>
-    <hyperlink ref="G26" r:id="rId13" xr:uid="{00000000-0004-0000-0B00-00000C000000}"/>
+    <hyperlink ref="G26" r:id="rId12" xr:uid="{00000000-0004-0000-0B00-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FBAECCD-A664-4798-A72B-8871055C7066}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.21875" style="25" customWidth="1"/>
+    <col min="2" max="3" width="18.88671875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="24.21875" style="25" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" style="25" customWidth="1"/>
+    <col min="6" max="6" width="17" style="25" customWidth="1"/>
+    <col min="7" max="7" width="17.21875" style="25" customWidth="1"/>
+    <col min="8" max="8" width="17.109375" style="25" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" style="25" customWidth="1"/>
+    <col min="10" max="10" width="33.77734375" style="25" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="25"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="I1" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2" s="26">
+        <v>1</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>